<commit_message>
Sync planning SharePoint : S14
</commit_message>
<xml_diff>
--- a/Plannings 2026 S14.xlsx
+++ b/Plannings 2026 S14.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cdalpes.sharepoint.com/sites/msteams_bd0f90/Documents partages/02. USP - TOS - General/RH/Plannings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="13" documentId="8_{150E33BF-47F0-4B68-8AA0-FBA696D166AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6A1E570E-3024-42B6-B1F7-2E6DA6078454}"/>
+  <xr:revisionPtr revIDLastSave="22" documentId="8_{150E33BF-47F0-4B68-8AA0-FBA696D166AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{43AAB536-26BF-4921-B8A8-A04C20079534}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="152">
   <si>
     <t>Mars-2026</t>
   </si>
@@ -382,9 +382,15 @@
     <t>PUJOL Mathieu</t>
   </si>
   <si>
+    <t>INVEN</t>
+  </si>
+  <si>
     <t>09:45/18:00</t>
   </si>
   <si>
+    <t>07:30/11:30</t>
+  </si>
+  <si>
     <t>17:30/18:45</t>
   </si>
   <si>
@@ -395,6 +401,9 @@
   </si>
   <si>
     <t>EDF-A</t>
+  </si>
+  <si>
+    <t>11:30/17:00</t>
   </si>
   <si>
     <t>18:45/22:45</t>
@@ -620,7 +629,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="26">
+  <borders count="34">
     <border>
       <left/>
       <right/>
@@ -941,11 +950,119 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="88">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1139,13 +1256,7 @@
     <xf numFmtId="0" fontId="10" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1154,7 +1265,52 @@
     <xf numFmtId="0" fontId="10" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1177,8 +1333,8 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFCCFFFF"/>
       <color rgb="FFCC99FF"/>
-      <color rgb="FFCCFFFF"/>
     </mruColors>
   </colors>
   <extLst>
@@ -4320,50 +4476,6 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>71</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>71</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="83" name="Picture 1" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000053000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="123825" cy="123825"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>71</xdr:row>
@@ -6345,6 +6457,53 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="12801600" y="12544425"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>73</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>73</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="35" name="Image 34" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C20438AB-D331-4320-8743-3CB6BED06766}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{965B5492-7230-45E4-ACAF-2849F9724C0E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9601200" y="14068425"/>
           <a:ext cx="123825" cy="123825"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -7642,10 +7801,10 @@
       <c r="D60" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="E60" s="68" t="s">
+      <c r="E60" s="66" t="s">
         <v>95</v>
       </c>
-      <c r="F60" s="65" t="s">
+      <c r="F60" s="71" t="s">
         <v>18</v>
       </c>
       <c r="G60" s="27" t="s">
@@ -7664,10 +7823,10 @@
       <c r="D61" s="26" t="s">
         <v>98</v>
       </c>
-      <c r="E61" s="69" t="s">
+      <c r="E61" s="67" t="s">
         <v>99</v>
       </c>
-      <c r="F61" s="67" t="s">
+      <c r="F61" s="72" t="s">
         <v>76</v>
       </c>
       <c r="G61" s="26" t="s">
@@ -7687,7 +7846,7 @@
       <c r="E62" s="64" t="s">
         <v>21</v>
       </c>
-      <c r="F62" s="67" t="s">
+      <c r="F62" s="72" t="s">
         <v>101</v>
       </c>
       <c r="G62" s="25" t="s">
@@ -7707,7 +7866,7 @@
       <c r="E63" s="70" t="s">
         <v>104</v>
       </c>
-      <c r="F63" s="67" t="s">
+      <c r="F63" s="72" t="s">
         <v>101</v>
       </c>
       <c r="G63" s="26" t="s">
@@ -7724,10 +7883,10 @@
       <c r="D64" s="29" t="s">
         <v>30</v>
       </c>
-      <c r="E64" s="64" t="s">
+      <c r="E64" s="68" t="s">
         <v>106</v>
       </c>
-      <c r="F64" s="67" t="s">
+      <c r="F64" s="72" t="s">
         <v>101</v>
       </c>
       <c r="G64" s="25" t="s">
@@ -7744,10 +7903,10 @@
       <c r="D65" s="31" t="s">
         <v>107</v>
       </c>
-      <c r="E65" s="66" t="s">
+      <c r="E65" s="69" t="s">
         <v>108</v>
       </c>
-      <c r="F65" s="67" t="s">
+      <c r="F65" s="72" t="s">
         <v>101</v>
       </c>
       <c r="G65" s="26" t="s">
@@ -7765,7 +7924,7 @@
       <c r="E66" s="64" t="s">
         <v>21</v>
       </c>
-      <c r="F66" s="67" t="s">
+      <c r="F66" s="72" t="s">
         <v>101</v>
       </c>
       <c r="G66" s="42" t="s">
@@ -7780,10 +7939,10 @@
         <v>92</v>
       </c>
       <c r="D67" s="31"/>
-      <c r="E67" s="66" t="s">
+      <c r="E67" s="65" t="s">
         <v>109</v>
       </c>
-      <c r="F67" s="67" t="s">
+      <c r="F67" s="72" t="s">
         <v>101</v>
       </c>
       <c r="G67" s="34" t="s">
@@ -7798,10 +7957,10 @@
         <v>21</v>
       </c>
       <c r="D68" s="31"/>
-      <c r="E68" s="66" t="s">
+      <c r="E68" s="65" t="s">
         <v>101</v>
       </c>
-      <c r="F68" s="67" t="s">
+      <c r="F68" s="72" t="s">
         <v>101</v>
       </c>
       <c r="G68" s="34"/>
@@ -7814,10 +7973,10 @@
         <v>111</v>
       </c>
       <c r="D69" s="30"/>
-      <c r="E69" s="66" t="s">
+      <c r="E69" s="65" t="s">
         <v>101</v>
       </c>
-      <c r="F69" s="67" t="s">
+      <c r="F69" s="72" t="s">
         <v>101</v>
       </c>
       <c r="G69" s="41"/>
@@ -7854,114 +8013,122 @@
       <c r="H71" s="13"/>
     </row>
     <row r="72" spans="1:8">
-      <c r="A72" s="48" t="s">
+      <c r="A72" s="73" t="s">
         <v>113</v>
       </c>
-      <c r="B72" s="8" t="s">
+      <c r="B72" s="74" t="s">
         <v>21</v>
       </c>
-      <c r="C72" s="8"/>
-      <c r="D72" s="8" t="s">
+      <c r="C72" s="74"/>
+      <c r="D72" s="75" t="s">
+        <v>114</v>
+      </c>
+      <c r="E72" s="74" t="s">
         <v>21</v>
       </c>
-      <c r="E72" s="8" t="s">
+      <c r="F72" s="74" t="s">
         <v>21</v>
       </c>
-      <c r="F72" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="G72" s="8" t="s">
+      <c r="G72" s="74" t="s">
         <v>59</v>
       </c>
-      <c r="H72" s="9"/>
+      <c r="H72" s="76"/>
     </row>
     <row r="73" spans="1:8">
-      <c r="A73" s="53"/>
+      <c r="A73" s="77"/>
       <c r="B73" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C73" s="1"/>
-      <c r="D73" s="1" t="s">
-        <v>114</v>
+      <c r="D73" s="67" t="s">
+        <v>116</v>
       </c>
       <c r="E73" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F73" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G73" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="H73" s="13"/>
+        <v>119</v>
+      </c>
+      <c r="H73" s="78"/>
     </row>
     <row r="74" spans="1:8">
-      <c r="A74" s="53"/>
+      <c r="A74" s="77"/>
       <c r="B74" s="1"/>
       <c r="C74" s="1"/>
-      <c r="D74" s="1"/>
+      <c r="D74" s="64" t="s">
+        <v>21</v>
+      </c>
       <c r="E74" s="20" t="s">
         <v>72</v>
       </c>
       <c r="F74" s="1"/>
       <c r="G74" s="25" t="s">
-        <v>118</v>
-      </c>
-      <c r="H74" s="13"/>
+        <v>120</v>
+      </c>
+      <c r="H74" s="78"/>
     </row>
     <row r="75" spans="1:8">
-      <c r="A75" s="53"/>
+      <c r="A75" s="77"/>
       <c r="B75" s="1"/>
       <c r="C75" s="1"/>
-      <c r="D75" s="1"/>
+      <c r="D75" s="65" t="s">
+        <v>121</v>
+      </c>
       <c r="E75" s="21" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="F75" s="1"/>
       <c r="G75" s="26" t="s">
-        <v>120</v>
-      </c>
-      <c r="H75" s="13"/>
+        <v>123</v>
+      </c>
+      <c r="H75" s="78"/>
     </row>
     <row r="76" spans="1:8">
-      <c r="A76" s="53"/>
+      <c r="A76" s="77"/>
       <c r="B76" s="1"/>
       <c r="C76" s="1"/>
-      <c r="D76" s="1"/>
+      <c r="D76" s="65" t="s">
+        <v>101</v>
+      </c>
       <c r="E76" s="21"/>
       <c r="F76" s="1"/>
       <c r="G76" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="H76" s="13"/>
-    </row>
-    <row r="77" spans="1:8" ht="15.75" thickBot="1">
-      <c r="A77" s="49"/>
-      <c r="B77" s="11"/>
-      <c r="C77" s="11"/>
-      <c r="D77" s="11"/>
-      <c r="E77" s="23"/>
-      <c r="F77" s="11"/>
-      <c r="G77" s="11" t="s">
-        <v>121</v>
-      </c>
-      <c r="H77" s="12"/>
+      <c r="H76" s="78"/>
+    </row>
+    <row r="77" spans="1:8">
+      <c r="A77" s="79"/>
+      <c r="B77" s="80"/>
+      <c r="C77" s="80"/>
+      <c r="D77" s="81" t="s">
+        <v>101</v>
+      </c>
+      <c r="E77" s="82"/>
+      <c r="F77" s="80"/>
+      <c r="G77" s="80" t="s">
+        <v>124</v>
+      </c>
+      <c r="H77" s="83"/>
     </row>
     <row r="78" spans="1:8">
-      <c r="A78" s="48" t="s">
-        <v>122</v>
-      </c>
-      <c r="B78" s="32" t="s">
+      <c r="A78" s="60" t="s">
+        <v>125</v>
+      </c>
+      <c r="B78" s="31" t="s">
         <v>34</v>
       </c>
-      <c r="C78" s="8"/>
-      <c r="D78" s="8"/>
-      <c r="E78" s="8"/>
-      <c r="F78" s="8"/>
-      <c r="G78" s="33" t="s">
+      <c r="C78" s="1"/>
+      <c r="D78" s="1"/>
+      <c r="E78" s="1"/>
+      <c r="F78" s="1"/>
+      <c r="G78" s="34" t="s">
         <v>8</v>
       </c>
-      <c r="H78" s="9"/>
+      <c r="H78" s="13"/>
     </row>
     <row r="79" spans="1:8">
       <c r="A79" s="53"/>
@@ -7997,13 +8164,13 @@
       <c r="E81" s="11"/>
       <c r="F81" s="11"/>
       <c r="G81" s="11" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="H81" s="12"/>
     </row>
     <row r="82" spans="1:8">
       <c r="A82" s="48" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="B82" s="8"/>
       <c r="C82" s="8"/>
@@ -8020,7 +8187,7 @@
       <c r="B83" s="11"/>
       <c r="C83" s="11"/>
       <c r="D83" s="28" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="E83" s="11"/>
       <c r="F83" s="11"/>
@@ -8029,7 +8196,7 @@
     </row>
     <row r="84" spans="1:8">
       <c r="A84" s="48" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="B84" s="8"/>
       <c r="C84" s="8"/>
@@ -8079,7 +8246,7 @@
     </row>
     <row r="88" spans="1:8" ht="15.75" thickBot="1">
       <c r="A88" s="14" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B88" s="50"/>
       <c r="C88" s="51"/>
@@ -8091,7 +8258,7 @@
     </row>
     <row r="89" spans="1:8">
       <c r="A89" s="60" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="B89" s="1"/>
       <c r="C89" s="1"/>
@@ -8116,16 +8283,16 @@
       </c>
       <c r="E90" s="11"/>
       <c r="F90" s="11" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="G90" s="11"/>
       <c r="H90" s="12" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
     </row>
     <row r="91" spans="1:8">
       <c r="A91" s="48" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="B91" s="8"/>
       <c r="C91" s="8"/>
@@ -8142,7 +8309,7 @@
       <c r="B92" s="11"/>
       <c r="C92" s="11"/>
       <c r="D92" s="28" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="E92" s="11"/>
       <c r="F92" s="11"/>
@@ -8204,12 +8371,12 @@
   <sheetData>
     <row r="1" spans="1:5" ht="15.75">
       <c r="A1" s="3" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="B4" s="62" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="C4" s="62"/>
       <c r="D4" s="62"/>
@@ -8217,7 +8384,7 @@
     </row>
     <row r="5" spans="1:5">
       <c r="B5" s="63" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C5" s="63"/>
       <c r="D5" s="63"/>
@@ -8228,32 +8395,32 @@
         <v>9</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="71">
-        <v>0</v>
-      </c>
-      <c r="C7" s="71">
-        <v>0</v>
-      </c>
-      <c r="D7" s="71">
-        <v>0</v>
-      </c>
-      <c r="E7" s="71">
+      <c r="B7" s="84">
+        <v>0</v>
+      </c>
+      <c r="C7" s="84">
+        <v>0</v>
+      </c>
+      <c r="D7" s="84">
+        <v>0</v>
+      </c>
+      <c r="E7" s="84">
         <v>0</v>
       </c>
     </row>
@@ -8261,16 +8428,16 @@
       <c r="A8" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="71">
-        <v>0</v>
-      </c>
-      <c r="C8" s="71">
-        <v>0</v>
-      </c>
-      <c r="D8" s="71">
-        <v>0</v>
-      </c>
-      <c r="E8" s="71">
+      <c r="B8" s="84">
+        <v>0</v>
+      </c>
+      <c r="C8" s="84">
+        <v>0</v>
+      </c>
+      <c r="D8" s="84">
+        <v>0</v>
+      </c>
+      <c r="E8" s="84">
         <v>0</v>
       </c>
     </row>
@@ -8278,16 +8445,16 @@
       <c r="A9" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="B9" s="71">
-        <v>0</v>
-      </c>
-      <c r="C9" s="71">
+      <c r="B9" s="84">
+        <v>0</v>
+      </c>
+      <c r="C9" s="84">
         <v>4.1667000000000003E-2</v>
       </c>
-      <c r="D9" s="71">
-        <v>0</v>
-      </c>
-      <c r="E9" s="71">
+      <c r="D9" s="84">
+        <v>0</v>
+      </c>
+      <c r="E9" s="84">
         <v>0</v>
       </c>
     </row>
@@ -8295,16 +8462,16 @@
       <c r="A10" s="24" t="s">
         <v>37</v>
       </c>
-      <c r="B10" s="71">
-        <v>0</v>
-      </c>
-      <c r="C10" s="71">
-        <v>0</v>
-      </c>
-      <c r="D10" s="71">
-        <v>0</v>
-      </c>
-      <c r="E10" s="71">
+      <c r="B10" s="84">
+        <v>0</v>
+      </c>
+      <c r="C10" s="84">
+        <v>0</v>
+      </c>
+      <c r="D10" s="84">
+        <v>0</v>
+      </c>
+      <c r="E10" s="84">
         <v>0</v>
       </c>
     </row>
@@ -8312,16 +8479,16 @@
       <c r="A11" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="B11" s="71">
-        <v>0</v>
-      </c>
-      <c r="C11" s="71">
-        <v>0</v>
-      </c>
-      <c r="D11" s="71">
-        <v>0</v>
-      </c>
-      <c r="E11" s="71">
+      <c r="B11" s="84">
+        <v>0</v>
+      </c>
+      <c r="C11" s="84">
+        <v>0</v>
+      </c>
+      <c r="D11" s="84">
+        <v>0</v>
+      </c>
+      <c r="E11" s="84">
         <v>0</v>
       </c>
     </row>
@@ -8329,16 +8496,16 @@
       <c r="A12" s="24" t="s">
         <v>40</v>
       </c>
-      <c r="B12" s="71">
-        <v>0</v>
-      </c>
-      <c r="C12" s="71">
-        <v>0</v>
-      </c>
-      <c r="D12" s="71">
-        <v>0</v>
-      </c>
-      <c r="E12" s="71">
+      <c r="B12" s="84">
+        <v>0</v>
+      </c>
+      <c r="C12" s="84">
+        <v>0</v>
+      </c>
+      <c r="D12" s="84">
+        <v>0</v>
+      </c>
+      <c r="E12" s="84">
         <v>0</v>
       </c>
     </row>
@@ -8346,16 +8513,16 @@
       <c r="A13" s="24" t="s">
         <v>45</v>
       </c>
-      <c r="B13" s="71">
-        <v>0</v>
-      </c>
-      <c r="C13" s="71">
-        <v>0</v>
-      </c>
-      <c r="D13" s="71">
+      <c r="B13" s="84">
+        <v>0</v>
+      </c>
+      <c r="C13" s="84">
+        <v>0</v>
+      </c>
+      <c r="D13" s="84">
         <v>0.24166699999999999</v>
       </c>
-      <c r="E13" s="71">
+      <c r="E13" s="84">
         <v>0</v>
       </c>
     </row>
@@ -8363,16 +8530,16 @@
       <c r="A14" s="24" t="s">
         <v>52</v>
       </c>
-      <c r="B14" s="71">
-        <v>0</v>
-      </c>
-      <c r="C14" s="71">
-        <v>0</v>
-      </c>
-      <c r="D14" s="71">
-        <v>0</v>
-      </c>
-      <c r="E14" s="71">
+      <c r="B14" s="84">
+        <v>0</v>
+      </c>
+      <c r="C14" s="84">
+        <v>0</v>
+      </c>
+      <c r="D14" s="84">
+        <v>0</v>
+      </c>
+      <c r="E14" s="84">
         <v>0</v>
       </c>
     </row>
@@ -8380,16 +8547,16 @@
       <c r="A15" s="24" t="s">
         <v>68</v>
       </c>
-      <c r="B15" s="71">
-        <v>0</v>
-      </c>
-      <c r="C15" s="71">
-        <v>0</v>
-      </c>
-      <c r="D15" s="71">
-        <v>0</v>
-      </c>
-      <c r="E15" s="71">
+      <c r="B15" s="84">
+        <v>0</v>
+      </c>
+      <c r="C15" s="84">
+        <v>0</v>
+      </c>
+      <c r="D15" s="84">
+        <v>0</v>
+      </c>
+      <c r="E15" s="84">
         <v>0</v>
       </c>
     </row>
@@ -8397,16 +8564,16 @@
       <c r="A16" s="24" t="s">
         <v>69</v>
       </c>
-      <c r="B16" s="71">
+      <c r="B16" s="84">
         <v>3.9584000000000001E-2</v>
       </c>
-      <c r="C16" s="71">
+      <c r="C16" s="84">
         <v>8.3334000000000005E-2</v>
       </c>
-      <c r="D16" s="71">
-        <v>0</v>
-      </c>
-      <c r="E16" s="71">
+      <c r="D16" s="84">
+        <v>0</v>
+      </c>
+      <c r="E16" s="84">
         <v>0</v>
       </c>
     </row>
@@ -8414,33 +8581,33 @@
       <c r="A17" s="24" t="s">
         <v>82</v>
       </c>
-      <c r="B17" s="71">
-        <v>0</v>
-      </c>
-      <c r="C17" s="71">
-        <v>0</v>
-      </c>
-      <c r="D17" s="71">
-        <v>0</v>
-      </c>
-      <c r="E17" s="71">
+      <c r="B17" s="84">
+        <v>0</v>
+      </c>
+      <c r="C17" s="84">
+        <v>0</v>
+      </c>
+      <c r="D17" s="84">
+        <v>0</v>
+      </c>
+      <c r="E17" s="84">
         <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" s="24" t="s">
-        <v>139</v>
-      </c>
-      <c r="B18" s="71">
-        <v>0</v>
-      </c>
-      <c r="C18" s="71">
-        <v>0</v>
-      </c>
-      <c r="D18" s="71">
-        <v>0</v>
-      </c>
-      <c r="E18" s="71">
+        <v>142</v>
+      </c>
+      <c r="B18" s="84">
+        <v>0</v>
+      </c>
+      <c r="C18" s="84">
+        <v>0</v>
+      </c>
+      <c r="D18" s="84">
+        <v>0</v>
+      </c>
+      <c r="E18" s="84">
         <v>0</v>
       </c>
     </row>
@@ -8448,16 +8615,16 @@
       <c r="A19" s="24" t="s">
         <v>83</v>
       </c>
-      <c r="B19" s="71">
-        <v>0</v>
-      </c>
-      <c r="C19" s="71">
-        <v>0</v>
-      </c>
-      <c r="D19" s="71">
-        <v>0</v>
-      </c>
-      <c r="E19" s="71">
+      <c r="B19" s="84">
+        <v>0</v>
+      </c>
+      <c r="C19" s="84">
+        <v>0</v>
+      </c>
+      <c r="D19" s="84">
+        <v>0</v>
+      </c>
+      <c r="E19" s="84">
         <v>0</v>
       </c>
     </row>
@@ -8465,16 +8632,16 @@
       <c r="A20" s="24" t="s">
         <v>84</v>
       </c>
-      <c r="B20" s="71">
-        <v>0</v>
-      </c>
-      <c r="C20" s="71">
-        <v>0</v>
-      </c>
-      <c r="D20" s="71">
-        <v>0</v>
-      </c>
-      <c r="E20" s="71">
+      <c r="B20" s="84">
+        <v>0</v>
+      </c>
+      <c r="C20" s="84">
+        <v>0</v>
+      </c>
+      <c r="D20" s="84">
+        <v>0</v>
+      </c>
+      <c r="E20" s="84">
         <v>0</v>
       </c>
     </row>
@@ -8482,16 +8649,16 @@
       <c r="A21" s="24" t="s">
         <v>85</v>
       </c>
-      <c r="B21" s="71">
-        <v>0</v>
-      </c>
-      <c r="C21" s="71">
-        <v>0</v>
-      </c>
-      <c r="D21" s="71">
-        <v>0</v>
-      </c>
-      <c r="E21" s="71">
+      <c r="B21" s="84">
+        <v>0</v>
+      </c>
+      <c r="C21" s="84">
+        <v>0</v>
+      </c>
+      <c r="D21" s="84">
+        <v>0</v>
+      </c>
+      <c r="E21" s="84">
         <v>0</v>
       </c>
     </row>
@@ -8499,33 +8666,33 @@
       <c r="A22" s="24" t="s">
         <v>86</v>
       </c>
-      <c r="B22" s="71">
-        <v>0</v>
-      </c>
-      <c r="C22" s="71">
-        <v>0</v>
-      </c>
-      <c r="D22" s="71">
-        <v>0</v>
-      </c>
-      <c r="E22" s="71">
+      <c r="B22" s="84">
+        <v>0</v>
+      </c>
+      <c r="C22" s="84">
+        <v>0</v>
+      </c>
+      <c r="D22" s="84">
+        <v>0</v>
+      </c>
+      <c r="E22" s="84">
         <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="24" t="s">
-        <v>140</v>
-      </c>
-      <c r="B23" s="71">
-        <v>0</v>
-      </c>
-      <c r="C23" s="71">
-        <v>0</v>
-      </c>
-      <c r="D23" s="71">
-        <v>0</v>
-      </c>
-      <c r="E23" s="71">
+        <v>143</v>
+      </c>
+      <c r="B23" s="84">
+        <v>0</v>
+      </c>
+      <c r="C23" s="84">
+        <v>0</v>
+      </c>
+      <c r="D23" s="84">
+        <v>0</v>
+      </c>
+      <c r="E23" s="84">
         <v>0</v>
       </c>
     </row>
@@ -8533,16 +8700,16 @@
       <c r="A24" s="24" t="s">
         <v>87</v>
       </c>
-      <c r="B24" s="71">
-        <v>0</v>
-      </c>
-      <c r="C24" s="71">
-        <v>0</v>
-      </c>
-      <c r="D24" s="71">
+      <c r="B24" s="84">
+        <v>0</v>
+      </c>
+      <c r="C24" s="84">
+        <v>0</v>
+      </c>
+      <c r="D24" s="84">
         <v>0.25</v>
       </c>
-      <c r="E24" s="71">
+      <c r="E24" s="84">
         <v>0</v>
       </c>
     </row>
@@ -8550,16 +8717,16 @@
       <c r="A25" s="24" t="s">
         <v>91</v>
       </c>
-      <c r="B25" s="71">
-        <v>0</v>
-      </c>
-      <c r="C25" s="71">
+      <c r="B25" s="84">
+        <v>0</v>
+      </c>
+      <c r="C25" s="84">
         <v>0.45833400000000002</v>
       </c>
-      <c r="D25" s="71">
-        <v>0</v>
-      </c>
-      <c r="E25" s="71">
+      <c r="D25" s="84">
+        <v>0</v>
+      </c>
+      <c r="E25" s="84">
         <v>0</v>
       </c>
     </row>
@@ -8567,16 +8734,16 @@
       <c r="A26" s="24" t="s">
         <v>94</v>
       </c>
-      <c r="B26" s="71">
-        <v>0</v>
-      </c>
-      <c r="C26" s="71">
+      <c r="B26" s="84">
+        <v>0</v>
+      </c>
+      <c r="C26" s="84">
         <v>0.16666700000000001</v>
       </c>
-      <c r="D26" s="71">
+      <c r="D26" s="84">
         <v>8.3334000000000005E-2</v>
       </c>
-      <c r="E26" s="71">
+      <c r="E26" s="84">
         <v>0</v>
       </c>
     </row>
@@ -8584,16 +8751,16 @@
       <c r="A27" s="24" t="s">
         <v>112</v>
       </c>
-      <c r="B27" s="71">
-        <v>0</v>
-      </c>
-      <c r="C27" s="71">
-        <v>0</v>
-      </c>
-      <c r="D27" s="71">
-        <v>0</v>
-      </c>
-      <c r="E27" s="71">
+      <c r="B27" s="84">
+        <v>0</v>
+      </c>
+      <c r="C27" s="84">
+        <v>0</v>
+      </c>
+      <c r="D27" s="84">
+        <v>0</v>
+      </c>
+      <c r="E27" s="84">
         <v>0</v>
       </c>
     </row>
@@ -8601,132 +8768,132 @@
       <c r="A28" s="24" t="s">
         <v>113</v>
       </c>
-      <c r="B28" s="71">
-        <v>0</v>
-      </c>
-      <c r="C28" s="71">
-        <v>0</v>
-      </c>
-      <c r="D28" s="71">
-        <v>0</v>
-      </c>
-      <c r="E28" s="71">
+      <c r="B28" s="84">
+        <v>0</v>
+      </c>
+      <c r="C28" s="84">
+        <v>0</v>
+      </c>
+      <c r="D28" s="84">
+        <v>0</v>
+      </c>
+      <c r="E28" s="84">
         <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="24" t="s">
-        <v>122</v>
-      </c>
-      <c r="B29" s="71">
-        <v>0</v>
-      </c>
-      <c r="C29" s="71">
+        <v>125</v>
+      </c>
+      <c r="B29" s="84">
+        <v>0</v>
+      </c>
+      <c r="C29" s="84">
         <v>0.125</v>
       </c>
-      <c r="D29" s="71">
+      <c r="D29" s="84">
         <v>0.159723</v>
       </c>
-      <c r="E29" s="71">
+      <c r="E29" s="84">
         <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="24" t="s">
-        <v>124</v>
-      </c>
-      <c r="B30" s="71">
-        <v>0</v>
-      </c>
-      <c r="C30" s="71">
-        <v>0</v>
-      </c>
-      <c r="D30" s="71">
-        <v>0</v>
-      </c>
-      <c r="E30" s="71">
+        <v>127</v>
+      </c>
+      <c r="B30" s="84">
+        <v>0</v>
+      </c>
+      <c r="C30" s="84">
+        <v>0</v>
+      </c>
+      <c r="D30" s="84">
+        <v>0</v>
+      </c>
+      <c r="E30" s="84">
         <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="24" t="s">
-        <v>126</v>
-      </c>
-      <c r="B31" s="71">
-        <v>0</v>
-      </c>
-      <c r="C31" s="71">
-        <v>0</v>
-      </c>
-      <c r="D31" s="71">
-        <v>0</v>
-      </c>
-      <c r="E31" s="71">
+        <v>129</v>
+      </c>
+      <c r="B31" s="84">
+        <v>0</v>
+      </c>
+      <c r="C31" s="84">
+        <v>0</v>
+      </c>
+      <c r="D31" s="84">
+        <v>0</v>
+      </c>
+      <c r="E31" s="84">
         <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:5">
       <c r="A32" s="24" t="s">
-        <v>127</v>
-      </c>
-      <c r="B32" s="71">
-        <v>0</v>
-      </c>
-      <c r="C32" s="71">
-        <v>0</v>
-      </c>
-      <c r="D32" s="71">
-        <v>0</v>
-      </c>
-      <c r="E32" s="71">
+        <v>130</v>
+      </c>
+      <c r="B32" s="84">
+        <v>0</v>
+      </c>
+      <c r="C32" s="84">
+        <v>0</v>
+      </c>
+      <c r="D32" s="84">
+        <v>0</v>
+      </c>
+      <c r="E32" s="84">
         <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:5">
       <c r="A33" s="24" t="s">
-        <v>128</v>
-      </c>
-      <c r="B33" s="71">
-        <v>0</v>
-      </c>
-      <c r="C33" s="71">
-        <v>0</v>
-      </c>
-      <c r="D33" s="71">
-        <v>0</v>
-      </c>
-      <c r="E33" s="71">
+        <v>131</v>
+      </c>
+      <c r="B33" s="84">
+        <v>0</v>
+      </c>
+      <c r="C33" s="84">
+        <v>0</v>
+      </c>
+      <c r="D33" s="84">
+        <v>0</v>
+      </c>
+      <c r="E33" s="84">
         <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:5">
       <c r="A34" s="24" t="s">
-        <v>131</v>
-      </c>
-      <c r="B34" s="71">
-        <v>0</v>
-      </c>
-      <c r="C34" s="71">
-        <v>0</v>
-      </c>
-      <c r="D34" s="71">
-        <v>0</v>
-      </c>
-      <c r="E34" s="71">
+        <v>134</v>
+      </c>
+      <c r="B34" s="84">
+        <v>0</v>
+      </c>
+      <c r="C34" s="84">
+        <v>0</v>
+      </c>
+      <c r="D34" s="84">
+        <v>0</v>
+      </c>
+      <c r="E34" s="84">
         <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:5">
-      <c r="B35" s="72">
+      <c r="B35" s="85">
         <v>3.9584000000000001E-2</v>
       </c>
-      <c r="C35" s="72">
+      <c r="C35" s="85">
         <v>0.875</v>
       </c>
-      <c r="D35" s="72">
+      <c r="D35" s="85">
         <v>0.73472300000000001</v>
       </c>
-      <c r="E35" s="72">
+      <c r="E35" s="85">
         <v>0</v>
       </c>
     </row>
@@ -8746,45 +8913,45 @@
   <sheetData>
     <row r="1" spans="1:2" ht="15.75">
       <c r="A1" s="3" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
     </row>
     <row r="4" spans="1:2">
-      <c r="A4" s="73" t="s">
-        <v>141</v>
-      </c>
-      <c r="B4" s="74" t="s">
-        <v>142</v>
+      <c r="A4" s="86" t="s">
+        <v>144</v>
+      </c>
+      <c r="B4" s="87" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="5" spans="1:2">
-      <c r="A5" s="73" t="s">
-        <v>143</v>
-      </c>
-      <c r="B5" s="74"/>
+      <c r="A5" s="86" t="s">
+        <v>146</v>
+      </c>
+      <c r="B5" s="87"/>
     </row>
     <row r="6" spans="1:2">
-      <c r="A6" s="73" t="s">
-        <v>144</v>
-      </c>
-      <c r="B6" s="74" t="s">
+      <c r="A6" s="86" t="s">
+        <v>147</v>
+      </c>
+      <c r="B6" s="87" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="7" spans="1:2">
-      <c r="A7" s="73" t="s">
-        <v>145</v>
-      </c>
-      <c r="B7" s="74" t="s">
-        <v>146</v>
+      <c r="A7" s="86" t="s">
+        <v>148</v>
+      </c>
+      <c r="B7" s="87" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="8" spans="1:2">
-      <c r="A8" s="73" t="s">
-        <v>147</v>
-      </c>
-      <c r="B8" s="74" t="s">
-        <v>148</v>
+      <c r="A8" s="86" t="s">
+        <v>150</v>
+      </c>
+      <c r="B8" s="87" t="s">
+        <v>151</v>
       </c>
     </row>
   </sheetData>

</xml_diff>